<commit_message>
updated data, added data existence file
</commit_message>
<xml_diff>
--- a/data/results of data sharing requests.xlsx
+++ b/data/results of data sharing requests.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Ian/git/repository-of-published-irap-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CA4D958-A2CE-F849-8C12-D45EF6BC0B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C95689FD-6523-E043-83D2-6DD8BEBC831B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="32780" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1654,7 +1654,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1677,12 +1677,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -2212,16 +2206,16 @@
       <c r="M3" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="N3" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="O3" s="10" t="s">
+      <c r="N3" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O3" s="4" t="s">
         <v>337</v>
       </c>
       <c r="P3" s="4" t="s">
         <v>306</v>
       </c>
-      <c r="Q3" s="9" t="b">
+      <c r="Q3" s="3" t="b">
         <v>0</v>
       </c>
       <c r="R3" s="3" t="s">
@@ -3007,13 +3001,13 @@
       <c r="L17" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="M17" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="N17" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="O17" s="10" t="s">
+      <c r="M17" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N17" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O17" s="4" t="s">
         <v>343</v>
       </c>
       <c r="P17" s="4" t="b">
@@ -3065,13 +3059,13 @@
       <c r="L18" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="M18" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="N18" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="O18" s="10" t="s">
+      <c r="M18" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N18" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O18" s="4" t="s">
         <v>343</v>
       </c>
       <c r="P18" s="4" t="b">
@@ -3295,10 +3289,10 @@
       <c r="L22" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="M22" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="N22" s="9" t="b">
+      <c r="M22" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N22" s="3" t="b">
         <v>0</v>
       </c>
       <c r="O22" s="4" t="s">
@@ -3352,10 +3346,10 @@
       <c r="L23" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="M23" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="N23" s="9" t="b">
+      <c r="M23" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N23" s="3" t="b">
         <v>0</v>
       </c>
       <c r="O23" s="4" t="s">
@@ -3409,10 +3403,10 @@
       <c r="L24" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="M24" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="N24" s="9" t="b">
+      <c r="M24" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N24" s="3" t="b">
         <v>0</v>
       </c>
       <c r="O24" s="4" t="s">
@@ -3466,10 +3460,10 @@
       <c r="L25" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="M25" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="N25" s="9" t="b">
+      <c r="M25" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N25" s="3" t="b">
         <v>0</v>
       </c>
       <c r="O25" s="4" t="s">
@@ -3811,16 +3805,16 @@
       <c r="M31" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="N31" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="O31" s="10" t="s">
+      <c r="N31" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O31" s="4" t="s">
         <v>333</v>
       </c>
       <c r="P31" s="4" t="s">
         <v>304</v>
       </c>
-      <c r="Q31" s="9" t="b">
+      <c r="Q31" s="3" t="b">
         <v>0</v>
       </c>
       <c r="R31" s="3" t="s">
@@ -3868,16 +3862,16 @@
       <c r="M32" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="N32" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="O32" s="10" t="s">
+      <c r="N32" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O32" s="4" t="s">
         <v>333</v>
       </c>
       <c r="P32" s="4" t="s">
         <v>290</v>
       </c>
-      <c r="Q32" s="9" t="b">
+      <c r="Q32" s="3" t="b">
         <v>0</v>
       </c>
       <c r="R32" s="3" t="s">
@@ -4036,7 +4030,7 @@
         <v>0</v>
       </c>
       <c r="N35" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O35" s="7" t="s">
         <v>295</v>
@@ -4592,10 +4586,10 @@
       <c r="L45" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="M45" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="N45" s="9" t="b">
+      <c r="M45" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="N45" s="3" t="b">
         <v>0</v>
       </c>
       <c r="O45" s="4" t="s">
@@ -4876,16 +4870,16 @@
       <c r="M50" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="N50" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="O50" s="10" t="s">
+      <c r="N50" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O50" s="4" t="s">
         <v>338</v>
       </c>
       <c r="P50" s="4" t="s">
         <v>307</v>
       </c>
-      <c r="Q50" s="9" t="b">
+      <c r="Q50" s="3" t="b">
         <v>0</v>
       </c>
       <c r="R50" s="3" t="s">
@@ -4933,16 +4927,16 @@
       <c r="M51" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="N51" s="9" t="b">
-        <v>0</v>
-      </c>
-      <c r="O51" s="10" t="s">
+      <c r="N51" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O51" s="4" t="s">
         <v>334</v>
       </c>
       <c r="P51" s="4" t="s">
         <v>289</v>
       </c>
-      <c r="Q51" s="9" t="b">
+      <c r="Q51" s="3" t="b">
         <v>0</v>
       </c>
       <c r="R51" s="3" t="s">

</xml_diff>